<commit_message>
FIX - fixes wrongly aligned COR panel
* updated version of coordinate spreadsheet from Erik
* ISSUE inconsistent paddle direction persists
</commit_message>
<xml_diff>
--- a/gaps-db/resources/master-spreadsheet/TOF_Paddle_Orientations.xlsx
+++ b/gaps-db/resources/master-spreadsheet/TOF_Paddle_Orientations.xlsx
@@ -7228,8 +7228,9 @@
       <c r="O117" s="29">
         <v>0.0</v>
       </c>
-      <c r="P117" s="39">
-        <v>140.93</v>
+      <c r="P117" s="36">
+        <f>P116 + SWITCH($I117,CONCATENATE("+",P$9), 1, CONCATENATE("-",P$9), -1, 0)*$K117 + SWITCH($J117,CONCATENATE("+",P$9), 1, CONCATENATE("-",P$9), -1, 0)*SWITCH(MOD($A117-$M117,2),1,1,0,-1)*$L117</f>
+        <v>209.91</v>
       </c>
       <c r="Q117" s="2">
         <v>1.005E8</v>
@@ -7279,16 +7280,15 @@
         <v>109</v>
       </c>
       <c r="N118" s="38">
-        <f t="shared" ref="N118:P118" si="106">N117 + SWITCH($I118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K118 + SWITCH($J118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A118-$M118,2),1,1,0,-1)*$L118</f>
+        <f t="shared" ref="N118:O118" si="106">N117 + SWITCH($I118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K118 + SWITCH($J118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A118-$M118,2),1,1,0,-1)*$L118</f>
         <v>117.61</v>
       </c>
       <c r="O118" s="28">
         <f t="shared" si="106"/>
         <v>0</v>
       </c>
-      <c r="P118" s="36">
-        <f t="shared" si="106"/>
-        <v>126.26</v>
+      <c r="P118" s="39">
+        <v>140.93</v>
       </c>
       <c r="Q118" s="2">
         <v>1.002009E8</v>
@@ -7347,7 +7347,7 @@
       </c>
       <c r="P119" s="36">
         <f t="shared" si="108"/>
-        <v>111.59</v>
+        <v>126.26</v>
       </c>
       <c r="Q119" s="2">
         <v>1.002008E8</v>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="P120" s="36">
         <f t="shared" si="109"/>
-        <v>96.92</v>
+        <v>111.59</v>
       </c>
       <c r="Q120" s="2">
         <v>1.002007E8</v>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="P121" s="36">
         <f t="shared" si="110"/>
-        <v>82.25</v>
+        <v>96.92</v>
       </c>
       <c r="Q121" s="2">
         <v>1.002006E8</v>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="P122" s="36">
         <f t="shared" si="111"/>
-        <v>67.58</v>
+        <v>82.25</v>
       </c>
       <c r="Q122" s="2">
         <v>1.002005E8</v>
@@ -7583,7 +7583,7 @@
       </c>
       <c r="P123" s="36">
         <f t="shared" si="112"/>
-        <v>52.91</v>
+        <v>67.58</v>
       </c>
       <c r="Q123" s="2">
         <v>1.002004E8</v>
@@ -7642,7 +7642,7 @@
       </c>
       <c r="P124" s="36">
         <f t="shared" si="113"/>
-        <v>38.24</v>
+        <v>52.91</v>
       </c>
       <c r="Q124" s="2">
         <v>1.002003E8</v>
@@ -7701,7 +7701,7 @@
       </c>
       <c r="P125" s="36">
         <f t="shared" si="114"/>
-        <v>23.57</v>
+        <v>38.24</v>
       </c>
       <c r="Q125" s="2">
         <v>1.002002E8</v>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="P126" s="36">
         <f t="shared" si="115"/>
-        <v>8.9</v>
+        <v>23.57</v>
       </c>
       <c r="Q126" s="2">
         <v>1.002001E8</v>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="P127" s="36">
         <f t="shared" si="116"/>
-        <v>-5.77</v>
+        <v>8.9</v>
       </c>
       <c r="Q127" s="2">
         <v>1.002E8</v>

</xml_diff>

<commit_message>
FIX - fix paddles once and for all?
* new iteration of coordinates and paddle mapping spreadsheets from
  the tof team
* should fix paddle 108 problem
</commit_message>
<xml_diff>
--- a/gaps-db/resources/master-spreadsheet/TOF_Paddle_Orientations.xlsx
+++ b/gaps-db/resources/master-spreadsheet/TOF_Paddle_Orientations.xlsx
@@ -7223,13 +7223,15 @@
         <v>103</v>
       </c>
       <c r="N117" s="38">
-        <v>118.31</v>
-      </c>
-      <c r="O117" s="29">
-        <v>0.0</v>
+        <f t="shared" ref="N117:P117" si="106">N116 + SWITCH($I117,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K117 + SWITCH($J117,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A117-$M117,2),1,1,0,-1)*$L117</f>
+        <v>167.4</v>
+      </c>
+      <c r="O117" s="28">
+        <f t="shared" si="106"/>
+        <v>-85.4</v>
       </c>
       <c r="P117" s="36">
-        <f>P116 + SWITCH($I117,CONCATENATE("+",P$9), 1, CONCATENATE("-",P$9), -1, 0)*$K117 + SWITCH($J117,CONCATENATE("+",P$9), 1, CONCATENATE("-",P$9), -1, 0)*SWITCH(MOD($A117-$M117,2),1,1,0,-1)*$L117</f>
+        <f t="shared" si="106"/>
         <v>209.91</v>
       </c>
       <c r="Q117" s="2">
@@ -7280,12 +7282,10 @@
         <v>109</v>
       </c>
       <c r="N118" s="38">
-        <f t="shared" ref="N118:O118" si="106">N117 + SWITCH($I118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K118 + SWITCH($J118,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A118-$M118,2),1,1,0,-1)*$L118</f>
-        <v>117.61</v>
-      </c>
-      <c r="O118" s="28">
-        <f t="shared" si="106"/>
-        <v>0</v>
+        <v>118.31</v>
+      </c>
+      <c r="O118" s="29">
+        <v>0.0</v>
       </c>
       <c r="P118" s="39">
         <v>140.93</v>
@@ -7339,7 +7339,7 @@
       </c>
       <c r="N119" s="38">
         <f t="shared" ref="N119:P119" si="108">N118 + SWITCH($I119,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K119 + SWITCH($J119,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A119-$M119,2),1,1,0,-1)*$L119</f>
-        <v>118.31</v>
+        <v>119.01</v>
       </c>
       <c r="O119" s="28">
         <f t="shared" si="108"/>
@@ -7398,7 +7398,7 @@
       </c>
       <c r="N120" s="38">
         <f t="shared" ref="N120:P120" si="109">N119 + SWITCH($I120,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K120 + SWITCH($J120,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A120-$M120,2),1,1,0,-1)*$L120</f>
-        <v>117.61</v>
+        <v>118.31</v>
       </c>
       <c r="O120" s="28">
         <f t="shared" si="109"/>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="N121" s="38">
         <f t="shared" ref="N121:P121" si="110">N120 + SWITCH($I121,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K121 + SWITCH($J121,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A121-$M121,2),1,1,0,-1)*$L121</f>
-        <v>118.31</v>
+        <v>119.01</v>
       </c>
       <c r="O121" s="28">
         <f t="shared" si="110"/>
@@ -7516,7 +7516,7 @@
       </c>
       <c r="N122" s="38">
         <f t="shared" ref="N122:P122" si="111">N121 + SWITCH($I122,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K122 + SWITCH($J122,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A122-$M122,2),1,1,0,-1)*$L122</f>
-        <v>117.61</v>
+        <v>118.31</v>
       </c>
       <c r="O122" s="28">
         <f t="shared" si="111"/>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="N123" s="38">
         <f t="shared" ref="N123:P123" si="112">N122 + SWITCH($I123,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K123 + SWITCH($J123,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A123-$M123,2),1,1,0,-1)*$L123</f>
-        <v>118.31</v>
+        <v>119.01</v>
       </c>
       <c r="O123" s="28">
         <f t="shared" si="112"/>
@@ -7634,7 +7634,7 @@
       </c>
       <c r="N124" s="38">
         <f t="shared" ref="N124:P124" si="113">N123 + SWITCH($I124,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K124 + SWITCH($J124,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A124-$M124,2),1,1,0,-1)*$L124</f>
-        <v>117.61</v>
+        <v>118.31</v>
       </c>
       <c r="O124" s="28">
         <f t="shared" si="113"/>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="N125" s="38">
         <f t="shared" ref="N125:P125" si="114">N124 + SWITCH($I125,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K125 + SWITCH($J125,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A125-$M125,2),1,1,0,-1)*$L125</f>
-        <v>118.31</v>
+        <v>119.01</v>
       </c>
       <c r="O125" s="28">
         <f t="shared" si="114"/>
@@ -7752,7 +7752,7 @@
       </c>
       <c r="N126" s="38">
         <f t="shared" ref="N126:P126" si="115">N125 + SWITCH($I126,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K126 + SWITCH($J126,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A126-$M126,2),1,1,0,-1)*$L126</f>
-        <v>117.61</v>
+        <v>118.31</v>
       </c>
       <c r="O126" s="28">
         <f t="shared" si="115"/>
@@ -7811,7 +7811,7 @@
       </c>
       <c r="N127" s="38">
         <f t="shared" ref="N127:P127" si="116">N126 + SWITCH($I127,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*$K127 + SWITCH($J127,CONCATENATE("+",N$9), 1, CONCATENATE("-",N$9), -1, 0)*SWITCH(MOD($A127-$M127,2),1,1,0,-1)*$L127</f>
-        <v>118.31</v>
+        <v>119.01</v>
       </c>
       <c r="O127" s="28">
         <f t="shared" si="116"/>

</xml_diff>